<commit_message>
B1: confirmar ENTR-01 con 3 frases verificadas
cotejo cumple en los 10 tramos
</commit_message>
<xml_diff>
--- a/07_Datos/datos_procesados/cotejo_B1_diferencias.xlsx
+++ b/07_Datos/datos_procesados/cotejo_B1_diferencias.xlsx
@@ -794,7 +794,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E201"/>
+  <dimension ref="A1:E204"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -832,83 +832,83 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
-        <is>
-          <t>ENTR-02</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>04:47</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>Bueno, este... tenemos un equipo de personas</t>
-        </is>
-      </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>este... tenemos un equipo de personas</t>
-        </is>
-      </c>
-      <c r="E2" s="3" t="inlineStr">
-        <is>
-          <t>omitida</t>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>ENTR-01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>07:03</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Entonces, eh cuando haces un un censo, después puedes planificar y y y ver los los resultados que vas a tener este a futuro</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Entonces, eh cuando haces un un censo, después puedes planificar y y y ver los los resultados que vas a tener este a futuro</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>confirmada sin diferencia</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>ENTR-02</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>06:27</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>Bueno, aquí dentro de de esto mmm ningún no hemos tenido</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>Bueno, aquí dentro de esto ningún problema hemos tenido</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>cambiada</t>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>ENTR-01</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>07:47</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>La dificultad es cuando la la la palma está un poco alta o o ya este no puedes este ver eh o visualizar bien este la flor</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>La dificultad es cuando la la la palma está un poco alta o o ya este no puedes este ver eh o visualizar bien este la flor</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>confirmada sin diferencia</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>ENTR-02</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>17:36</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>La polinización en el híbrido es obligatoria</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>La polinización en híbridos es obligatoria</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>cambiada</t>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>ENTR-01</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>08:21</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Este sí, eh hay variedades, ¿no? Y de acuerdo a las variedades este son sus rendimientos.</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Este sí, eh hay variedades, ¿no? Y de acuerdo a las variedades este son sus rendimientos.</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>confirmada sin diferencia</t>
         </is>
       </c>
     </row>
@@ -920,17 +920,17 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>19:18</t>
+          <t>04:47</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Una planta adulta de palma africana o híbrido en pleno verano necesita entre 150 a 200 litros</t>
+          <t>Bueno, este... tenemos un equipo de personas</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Una planta adulta de palma africana necesita entre 150 a 200 litros</t>
+          <t>este... tenemos un equipo de personas</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
@@ -947,22 +947,22 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>23:29</t>
+          <t>06:27</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Bueno, creo que eso sería todo para la entrevista. Muchas gracias por su tiempo.</t>
+          <t>Bueno, aquí dentro de de esto mmm ningún no hemos tenido</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Bueno, creo que eso sería todo. Muchas gracias por su tiempo.</t>
+          <t>Bueno, aquí dentro de esto ningún problema hemos tenido</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>omitida</t>
+          <t>cambiada</t>
         </is>
       </c>
     </row>
@@ -974,44 +974,44 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>23:36</t>
+          <t>17:36</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>El pico de producción generalmente coincide con los meses posteriores al invierno</t>
+          <t>La polinización en el híbrido es obligatoria</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>El pico de producción coincide con los meses posteriores al invierno</t>
+          <t>La polinización en híbridos es obligatoria</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>omitida</t>
+          <t>cambiada</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>ENTR-03</t>
+          <t>ENTR-02</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>02:05</t>
+          <t>19:18</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Ya. El momento adecuado es cuando las flores...</t>
+          <t>Una planta adulta de palma africana o híbrido en pleno verano necesita entre 150 a 200 litros</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>El momento adecuado es cuando las flores...</t>
+          <t>Una planta adulta de palma africana necesita entre 150 a 200 litros</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -1023,49 +1023,49 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>ENTR-03</t>
+          <t>ENTR-02</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>03:10</t>
+          <t>23:29</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>El clima influye porque la palma necesita horas luz...</t>
+          <t>Bueno, creo que eso sería todo para la entrevista. Muchas gracias por su tiempo.</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>El clima influye porque la palma necesita horas de luz...</t>
+          <t>Bueno, creo que eso sería todo. Muchas gracias por su tiempo.</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>agregada</t>
+          <t>omitida</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>ENTR-03</t>
+          <t>ENTR-02</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>04:03</t>
+          <t>23:36</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Ya. Bueno, esto ha sido el tema sobre la polinización...</t>
+          <t>El pico de producción generalmente coincide con los meses posteriores al invierno</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>Bueno, esto ha sido el tema sobre la polinización</t>
+          <t>El pico de producción coincide con los meses posteriores al invierno</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
@@ -1077,22 +1077,22 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>ENTR-04</t>
+          <t>ENTR-03</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>04:19</t>
+          <t>02:05</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Normalmente nosotros cuando tenemos estos problemas, actuamos un mes antes realizando visitas a campo</t>
+          <t>Ya. El momento adecuado es cuando las flores...</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>Normalmente nosotros cuando tenemos estos problemas actuamos realizando visitas a campo</t>
+          <t>El momento adecuado es cuando las flores...</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
@@ -1104,211 +1104,211 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>ENTR-04</t>
+          <t>ENTR-03</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>05:08</t>
+          <t>03:10</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>En sí, no tenemos establecido un plazo máximo.</t>
+          <t>El clima influye porque la palma necesita horas luz...</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>En sí, no tenemos un plazo máximo definido.</t>
+          <t>El clima influye porque la palma necesita horas de luz...</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>cambiada</t>
+          <t>agregada</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>ENTR-04</t>
+          <t>ENTR-03</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>05:50</t>
+          <t>04:03</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>de que tiene muchos antioxidantes</t>
+          <t>Ya. Bueno, esto ha sido el tema sobre la polinización...</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>de que tiene bastantes antioxidantes</t>
+          <t>Bueno, esto ha sido el tema sobre la polinización</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>cambiada</t>
+          <t>omitida</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>ENTR-05</t>
+          <t>ENTR-04</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>00:28</t>
+          <t>04:19</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>Porque cuando se inició aquí [así transcrito por la app; posible error de reconocimiento de voz, verificar contra el audio] estaba pequeña</t>
+          <t>Normalmente nosotros cuando tenemos estos problemas, actuamos un mes antes realizando visitas a campo</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>porque cuando la finca inició estaba pequeña</t>
+          <t>Normalmente nosotros cuando tenemos estos problemas actuamos realizando visitas a campo</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>agregada</t>
+          <t>omitida</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>ENTR-05</t>
+          <t>ENTR-04</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>01:47</t>
+          <t>05:08</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>Ese conteo se le entrega en la tarde</t>
+          <t>En sí, no tenemos establecido un plazo máximo.</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>Ese conteo se entrega en la tarde</t>
+          <t>En sí, no tenemos un plazo máximo definido.</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>agregada</t>
+          <t>cambiada</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>ENTR-05</t>
+          <t>ENTR-04</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>03:04</t>
+          <t>05:50</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>Ahí le avisamos al encargado [así transcrito por la app; posible error de reconocimiento, verificar contra el audio], nosotros le damos el aviso.</t>
+          <t>de que tiene muchos antioxidantes</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>Ahí le avisamos al encargado, nosotros le damos el aviso...</t>
+          <t>de que tiene bastantes antioxidantes</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>agregada</t>
+          <t>cambiada</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>ENTR-06</t>
+          <t>ENTR-05</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>00:16</t>
+          <t>00:28</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>Yo tengo tres meses haciendo labor en lo que es chapea y [así transcrito por la app; posible error de reconocimiento, verificar contra el audio: "fútbol"].</t>
+          <t>Porque cuando se inició aquí [así transcrito por la app; posible error de reconocimiento de voz, verificar contra el audio] estaba pequeña</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>en lo que es chapea y fúmigo</t>
+          <t>porque cuando la finca inició estaba pequeña</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>cambiada</t>
+          <t>agregada</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>ENTR-06</t>
+          <t>ENTR-05</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>01:32</t>
+          <t>01:47</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>¿Alguna vez ha perdido el conteo o ha perdido la voz?</t>
+          <t>Ese conteo se le entrega en la tarde</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>¿Alguna vez ha perdido el conteo o se ha equivocado?</t>
+          <t>Ese conteo se entrega en la tarde</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>cambiada</t>
+          <t>agregada</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>ENTR-07</t>
+          <t>ENTR-05</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>00:56</t>
+          <t>03:04</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>Bueno, la libreta realmente la lleva al jefe de campo</t>
+          <t>Ahí le avisamos al encargado [así transcrito por la app; posible error de reconocimiento, verificar contra el audio], nosotros le damos el aviso.</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>Bueno, la libreta la lleva el jefe de campo</t>
+          <t>Ahí le avisamos al encargado, nosotros le damos el aviso...</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
@@ -1320,103 +1320,103 @@
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>ENTR-07</t>
+          <t>ENTR-06</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>01:40</t>
+          <t>00:16</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>Por lo general nada, pero diría que los seguimientos, que no suelen llegar los reportes...</t>
+          <t>Yo tengo tres meses haciendo labor en lo que es chapea y [así transcrito por la app; posible error de reconocimiento, verificar contra el audio: "fútbol"].</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>Por lo general nada, pero diría que los seguimientos...</t>
+          <t>en lo que es chapea y fúmigo</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>agregada</t>
+          <t>cambiada</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>ENTR-07</t>
+          <t>ENTR-06</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>02:41</t>
+          <t>01:32</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>Me suelen avisar inmediatamente por whatsapp...</t>
+          <t>¿Alguna vez ha perdido el conteo o ha perdido la voz?</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>Me suelen avisar por whatsapp...</t>
+          <t>¿Alguna vez ha perdido el conteo o se ha equivocado?</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>agregada</t>
+          <t>cambiada</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>ENTR-08</t>
+          <t>ENTR-07</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>06:15</t>
+          <t>00:56</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>En sí nosotros vemos si no hay desprendimiento, eso lo nosotros nos damos cuenta de que el fruto está verde.</t>
+          <t>Bueno, la libreta realmente la lleva al jefe de campo</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>En sí nosotros vemos si no hay desprendimiento, ahí nos damos cuenta...</t>
+          <t>Bueno, la libreta la lleva el jefe de campo</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>cambiada</t>
+          <t>agregada</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>ENTR-08</t>
+          <t>ENTR-07</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>06:31</t>
+          <t>01:40</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>Te puedo decir como que primero observar bien la la parte basal...</t>
+          <t>Por lo general nada, pero diría que los seguimientos, que no suelen llegar los reportes...</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>Primero observar bien la parte basal de la planta...</t>
+          <t>Por lo general nada, pero diría que los seguimientos...</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
@@ -1428,50 +1428,110 @@
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
+          <t>ENTR-07</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>02:41</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>Me suelen avisar inmediatamente por whatsapp...</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>Me suelen avisar por whatsapp...</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>agregada</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
           <t>ENTR-08</t>
         </is>
       </c>
-      <c r="B24" s="3" t="inlineStr">
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>06:15</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>En sí nosotros vemos si no hay desprendimiento, eso lo nosotros nos damos cuenta de que el fruto está verde.</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>En sí nosotros vemos si no hay desprendimiento, ahí nos damos cuenta...</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>cambiada</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>ENTR-08</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>06:31</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>Te puedo decir como que primero observar bien la la parte basal...</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>Primero observar bien la parte basal de la planta...</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>agregada</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>ENTR-08</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
         <is>
           <t>08:08</t>
         </is>
       </c>
-      <c r="C24" s="3" t="inlineStr">
+      <c r="C27" s="3" t="inlineStr">
         <is>
           <t>Y si usted utilizara una aplicación mediante una foto y y para es que mediante esa foto...</t>
         </is>
       </c>
-      <c r="D24" s="3" t="inlineStr">
+      <c r="D27" s="3" t="inlineStr">
         <is>
           <t>Y si usted utilizara una aplicación mediante una foto...</t>
         </is>
       </c>
-      <c r="E24" s="3" t="inlineStr">
+      <c r="E27" s="3" t="inlineStr">
         <is>
           <t>agregada</t>
         </is>
       </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="3" t="n"/>
-      <c r="B25" s="3" t="n"/>
-      <c r="C25" s="3" t="n"/>
-      <c r="D25" s="3" t="n"/>
-      <c r="E25" s="3" t="n"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="3" t="n"/>
-      <c r="B26" s="3" t="n"/>
-      <c r="C26" s="3" t="n"/>
-      <c r="D26" s="3" t="n"/>
-      <c r="E26" s="3" t="n"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="3" t="n"/>
-      <c r="B27" s="3" t="n"/>
-      <c r="C27" s="3" t="n"/>
-      <c r="D27" s="3" t="n"/>
-      <c r="E27" s="3" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="3" t="n"/>
@@ -2690,6 +2750,27 @@
       <c r="C201" s="3" t="n"/>
       <c r="D201" s="3" t="n"/>
       <c r="E201" s="3" t="n"/>
+    </row>
+    <row r="202">
+      <c r="A202" s="3" t="n"/>
+      <c r="B202" s="3" t="n"/>
+      <c r="C202" s="3" t="n"/>
+      <c r="D202" s="3" t="n"/>
+      <c r="E202" s="3" t="n"/>
+    </row>
+    <row r="203">
+      <c r="A203" s="3" t="n"/>
+      <c r="B203" s="3" t="n"/>
+      <c r="C203" s="3" t="n"/>
+      <c r="D203" s="3" t="n"/>
+      <c r="E203" s="3" t="n"/>
+    </row>
+    <row r="204">
+      <c r="A204" s="3" t="n"/>
+      <c r="B204" s="3" t="n"/>
+      <c r="C204" s="3" t="n"/>
+      <c r="D204" s="3" t="n"/>
+      <c r="E204" s="3" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>